<commit_message>
feat: remove safe storage and lose all held items on defeat
</commit_message>
<xml_diff>
--- a/config/excel/CfgCollections.xlsx
+++ b/config/excel/CfgCollections.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CfgCollections" sheetId="1" r:id="R23f52d2ea0994f60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CfgCollections" sheetId="1" r:id="R941d979d1ead4138"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -346,9 +346,7 @@
       <x:c r="G1" s="5" t="str">
         <x:v>Quality</x:v>
       </x:c>
-      <x:c r="H1" s="5" t="str">
-        <x:v>SafeAllowed</x:v>
-      </x:c>
+      <x:c r="H1"/>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
@@ -372,9 +370,7 @@
       <x:c r="G2" s="6" t="str">
         <x:v>int</x:v>
       </x:c>
-      <x:c r="H2" s="6" t="str">
-        <x:v>bool</x:v>
-      </x:c>
+      <x:c r="H2"/>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="8" t="str">
@@ -398,9 +394,7 @@
       <x:c r="G3" s="8" t="str">
         <x:v>品质</x:v>
       </x:c>
-      <x:c r="H3" s="8" t="str">
-        <x:v>是否允许安全箱保护</x:v>
-      </x:c>
+      <x:c r="H3"/>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="9" t="str">
@@ -424,9 +418,7 @@
       <x:c r="G4" s="9" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H4" s="10" t="b">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="H4"/>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="9" t="str">
@@ -450,9 +442,7 @@
       <x:c r="G5" s="9" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H5" s="10" t="b">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="H5"/>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="9" t="str">
@@ -476,9 +466,7 @@
       <x:c r="G6" s="9" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H6" s="10" t="b">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="H6"/>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
       <x:c r="A7" s="9" t="str">
@@ -502,9 +490,7 @@
       <x:c r="G7" s="9" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H7" s="10" t="b">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="H7"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>